<commit_message>
improve templates and examples
</commit_message>
<xml_diff>
--- a/data/Bioerosion_Data_TEMPLATE.xlsx
+++ b/data/Bioerosion_Data_TEMPLATE.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\__git\CBuRT\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp.sharepoint.com/sites/usgs-carbonate_budget_restoration_tool/Shared Documents/Carbonate Budget Tool Collaboration/Carbonate_Budget_Tool_Code/CarbonateBudgetRestorationTool_archive/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45902990-E8D2-4A36-811D-67E6EF519CF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{45902990-E8D2-4A36-811D-67E6EF519CF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{290E311F-34FF-4E05-863D-0F99766AABEE}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="3" xr2:uid="{19050643-5FB9-4299-B24C-C8F9EBB4329D}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="3" xr2:uid="{19050643-5FB9-4299-B24C-C8F9EBB4329D}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="4" r:id="rId1"/>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="32">
   <si>
     <t>Taxon</t>
   </si>
@@ -167,6 +167,12 @@
   </si>
   <si>
     <t>Survey_Area_Sponges_m2</t>
+  </si>
+  <si>
+    <t>Years_Post_Restoration</t>
+  </si>
+  <si>
+    <t>•  Input the monitoring timepoint in Years_Post_Restoration; months should be entered as fractional years, e.g., 3 months post outplanting = 0.25 y; pre-retoration data should be entered as -1</t>
   </si>
 </sst>
 </file>
@@ -237,11 +243,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -576,7 +583,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B1F19CC-78B5-4ED5-B7BB-7FAE8CE47042}">
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.45">
@@ -604,78 +611,83 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A7" s="3" t="s">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A8" s="3" t="s">
         <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A14" s="3" t="s">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A15" s="3" t="s">
         <v>16</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A15" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A20" s="3" t="s">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A21" s="3" t="s">
         <v>25</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A21" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A24" t="s">
         <v>28</v>
       </c>
     </row>
@@ -686,18 +698,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{097E6DCD-54F5-455D-97A6-7DF865AB568B}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="13.1328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.796875" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.53125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="5.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="23.265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -715,6 +727,9 @@
       </c>
       <c r="F1" t="s">
         <v>21</v>
+      </c>
+      <c r="G1" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -736,17 +751,17 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8E39944-BDAF-42EC-B85D-250380458002}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="13.1328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.73046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.73046875" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="5.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21.53125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -761,6 +776,9 @@
       </c>
       <c r="E1" t="s">
         <v>22</v>
+      </c>
+      <c r="F1" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -768,7 +786,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C1048576" xr:uid="{20125FB6-2368-4231-BA26-450E353A76B7}">
       <formula1>"0-20, 20-40, 40-60, 60-80, 80-100"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B1048576 B2" xr:uid="{2223DC14-4EAE-4087-A2E5-F0D15F10AA0B}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B1048576" xr:uid="{2223DC14-4EAE-4087-A2E5-F0D15F10AA0B}">
       <formula1>"Diadema antillarum, Echinometra lucunter, Echinometra viridis, Eucidaris tribuloides"</formula1>
     </dataValidation>
   </dataValidations>
@@ -778,7 +796,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14DD8175-6759-45E8-954F-11EB0116619A}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="13.1328125" bestFit="1" customWidth="1"/>
@@ -787,7 +805,7 @@
     <col min="4" max="4" width="22.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -800,10 +818,13 @@
       <c r="D1" t="s">
         <v>29</v>
       </c>
+      <c r="E1" t="s">
+        <v>30</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B1048576 B2" xr:uid="{145A3965-54F2-4637-AAFD-B7BE6990F686}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B1048576" xr:uid="{145A3965-54F2-4637-AAFD-B7BE6990F686}">
       <formula1>"Cliona aprica, Cliona caribbaea, Cliona tenuis, Cliona varians, Cliona delitrix, Siphonodictyon spp."</formula1>
     </dataValidation>
   </dataValidations>
@@ -812,28 +833,8 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="797e7fd4-719a-42b3-b312-968ffa9058ad">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="811eef35-9bdd-441e-81aa-50455f68c6c3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000AA90A7536739341825FB392424435FB" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ca57789ecb406bb7a99068f68ac4c0ed">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="797e7fd4-719a-42b3-b312-968ffa9058ad" xmlns:ns3="811eef35-9bdd-441e-81aa-50455f68c6c3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="89dc4794f4784a0bac47690674a3da53" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000AA90A7536739341825FB392424435FB" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="647735499ae6baa62e6fc7f5ed3567b4">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="797e7fd4-719a-42b3-b312-968ffa9058ad" xmlns:ns3="811eef35-9bdd-441e-81aa-50455f68c6c3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="47ff4a2bf1fedf465812d90a21a07c12" ns2:_="" ns3:_="">
     <xsd:import namespace="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
     <xsd:import namespace="811eef35-9bdd-441e-81aa-50455f68c6c3"/>
     <xsd:element name="properties">
@@ -1026,27 +1027,28 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="797e7fd4-719a-42b3-b312-968ffa9058ad">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="811eef35-9bdd-441e-81aa-50455f68c6c3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A206479D-07AC-477F-8545-4966E63B8E30}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0FB6342C-EC7C-49F8-97E7-6339AB75B937}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
-    <ds:schemaRef ds:uri="811eef35-9bdd-441e-81aa-50455f68c6c3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A81EFD0C-A7A2-40CC-AF34-FA5F0D62D046}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0AC9D92C-6A9E-424D-BBA1-C74B9FBA6A28}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
@@ -1064,6 +1066,25 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A206479D-07AC-477F-8545-4966E63B8E30}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0FB6342C-EC7C-49F8-97E7-6339AB75B937}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
+    <ds:schemaRef ds:uri="811eef35-9bdd-441e-81aa-50455f68c6c3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{6dd02d64-b7f3-43f7-a145-cfd68d338edf}" enabled="1" method="Standard" siteId="{0693b5ba-4b18-4d7b-9341-f32f400a5494}" removed="0"/>

</xml_diff>